<commit_message>
balance: niches for Power Charge, Accelerator, Shadow Clone and more
Power Charge 1.13 - 1.40 (the charged blow x2.13 - x2.4), Accelerator 10 - 15% for 4 turns, Shadow Clone one turn longer, Prism Dawn x1.4 power, Oracles' Action x1.5 (rows V001 - V030, D061 - D070). Measured before building with skill-battery variants and class-search compare=variant (C34, C38: no dominant party). The box of Power Charge shows the multiple it gives in both variants (it showed the stored value). Curve 36 of 44 within: C19 sits on the edge with or without these rows (400 battles: 6.51 against 6.53).
</commit_message>
<xml_diff>
--- a/data_tables/balance_skill_text.xlsx
+++ b/data_tables/balance_skill_text.xlsx
@@ -574,13 +574,13 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>ATK: 252% (+4-10%/Lv) -&gt; 314%   |   Paralysis: 30% (+3-5%/Lv) -&gt; 64% (L10)
+          <t>ATK: 328% (+6-15%/Lv) -&gt; 421%   |   Paralysis: 30% (+3-5%/Lv) -&gt; 64% (L10)
 Turns: 5 (Lv1-4) -&gt; 6 (Lv5-8) -&gt; 7 (Lv9-10)  |  TP Cost: 24 -&gt; 48  |  Speed: 1.1x</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Rows D041 - D080: power of Oracles' Action, life, speed</t>
+          <t>Rows D041 - D080: power of Oracles' Action (x1.5 more on 2026-10-16), life, speed</t>
         </is>
       </c>
     </row>
@@ -1116,12 +1116,12 @@
       <c r="E22" t="inlineStr">
         <is>
           <t>Number of dodges: 1 -&gt; 2 -&gt; 3 -&gt; 4 -&gt; 5 (L1-5 Max)   |   Chant: 0.75x
-Turns: 3 -&gt; 3 -&gt; 4 -&gt; 4 -&gt; 5   |   TP Cost: 17 -&gt; 20 -&gt; 24 -&gt; 28 -&gt; 33   |   Speed: 0.85x</t>
+Turns: 4 -&gt; 4 -&gt; 5 -&gt; 5 -&gt; 6   |   TP Cost: 17 -&gt; 20 -&gt; 24 -&gt; 28 -&gt; 33   |   Speed: 0.85x</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Rows K001: the generated box fell back to "Number of dodges UP"</t>
+          <t>Rows K001, V016 - V020 (one more turn): the generated box fell back to "Number of dodges UP"</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
balance: Kunoichi scrolls as her answer to armoured bosses
The late bosses are immune to her ailments and Shadow Sew needs a lower
level target; her scrolls deal a share of max HP, which ignores DEF.
Damage cap of the five element scrolls x3 (250-500 to 750-1500) and the
DEF debuff of Earth Scroll to -15% to -30%; texts of the three
hand-worded boxes updated.

Class-search: Kunoichi at C33 (Iron Fortress, DEF x3) 28% to 36%; no
other boss moved; the class stays in the band (64%). Higher caps, AGI or
ATK did not move C36 - C40. Full suite 9 of 9 steps.
</commit_message>
<xml_diff>
--- a/data_tables/balance_skill_text.xlsx
+++ b/data_tables/balance_skill_text.xlsx
@@ -687,12 +687,12 @@
       <c r="E7" t="inlineStr">
         <is>
           <t>Max HP damage: 6% -&gt; 7% -&gt; 9% -&gt; 10% -&gt; 12% (L1-5 Max)   |   Accuracy: 64% (+4%/Lv)
-ATK: -6% -&gt; -12% (3 Turns) | Damage cap: 250 -&gt; 500 | TP Cost: 20 (+2-3/Lv) -&gt; 30</t>
+ATK: -6% -&gt; -12% (3 Turns) | Damage cap: 750 -&gt; 1500 | TP Cost: 20 (+2-3/Lv) -&gt; 30</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Rows C068, A139, X001</t>
+          <t>Rows C068, A139, X001, K124-K157</t>
         </is>
       </c>
     </row>
@@ -715,12 +715,12 @@
       <c r="E8" t="inlineStr">
         <is>
           <t>Max HP damage: 6% -&gt; 7% -&gt; 9% -&gt; 10% -&gt; 12% (L1-5 Max)   |   Accuracy: 64% (+4%/Lv)
-Evasion: -10% -&gt; -23% (3 Turns) | Damage cap: 250 -&gt; 500 | TP Cost: 20 (+2-3/Lv) -&gt; 30</t>
+Evasion: -10% -&gt; -23% (3 Turns) | Damage cap: 750 -&gt; 1500 | TP Cost: 20 (+2-3/Lv) -&gt; 30</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Rows C165, A149, X011</t>
+          <t>Rows C165, A149, X011, K124-K157</t>
         </is>
       </c>
     </row>
@@ -743,12 +743,12 @@
       <c r="E9" t="inlineStr">
         <is>
           <t>Max HP damage: 6% -&gt; 7% -&gt; 9% -&gt; 10% -&gt; 12% (L1-5 Max)   |   Accuracy: 64% (+4%/Lv)
-DEF: -6% -&gt; -12% (3 Turns) | Damage cap: 250 -&gt; 500 | TP Cost: 20 (+2-3/Lv) -&gt; 30</t>
+DEF: -15% -&gt; -30% (3 Turns) | Damage cap: 750 -&gt; 1500 | TP Cost: 20 (+2-3/Lv) -&gt; 30</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Rows C064, A154, X016</t>
+          <t>Rows C064, A154, X016, K124-K157</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
balance: Accelerator and Amplify to all allies, Aim adds critical rate
Accelerator hits all allies, +27% to +40% speed for 8 turns; Amplify hits all allies; Aim adds 3 to 30 points of critical rate. One-skill trials, 16 bosses, 1000 battles each: Accelerator wins -4.9 > +0.6 and won fights 41% longer > 2.9% shorter; Amplify wins +0.2 > +1.1, cells hurt 4 > 0; Aim cells hurt 8 > 3. Skill battery hurt share: Accelerator 50% > 11%, Amplify 33% > 7%, Aim 26% > 21%.
</commit_message>
<xml_diff>
--- a/data_tables/balance_skill_text.xlsx
+++ b/data_tables/balance_skill_text.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1185,6 +1185,93 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Technique</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>TechniqueSkillData_0035.bin</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Aim</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Increase own accuracy and critical rate.</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Accuracy: +15% (+1-2%/Lv) -&gt; +30%   |   Critical rate: +3% (+3%/Lv) -&gt; +30% (L10)
+Turns: 5 -&gt; 9   |   TP Cost: 5 (+2-3/Lv) -&gt; 28</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Row Y022: effect 31 added, 3 points of critical rate a level</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Magic</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>MagicSkillData_0197.bin</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Accelerator</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Raise the party's speed.</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Rows V006 - V015, Y020: all allies, 27% - 40%, 8 turns</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Magic</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>MagicSkillData_0198.bin</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Amplify</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Raise the party's max HP.</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Row Y021: all allies</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
balance: Aim multiplies damage +10% to +30% instead of crit
Aim keeps its accuracy and gains the damage multiplier of Power Charge
(effect 191, +10% at level 1 to +30% at level 10) in place of the
critical rate. 16 bosses, 1000 battles each: wins +0.5, won fights
7.3% shorter, 0 hurt cells, 14 served. The shooter role keeps Aim up
(policy row). Battery: Aim hurt 21% to 6%, serve 2% to 13%.
</commit_message>
<xml_diff>
--- a/data_tables/balance_skill_text.xlsx
+++ b/data_tables/balance_skill_text.xlsx
@@ -1203,18 +1203,18 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Increase own accuracy and critical rate.</t>
+          <t>Increase own accuracy and physical damage.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Accuracy: +15% (+1-2%/Lv) -&gt; +30%   |   Critical rate: +3% (+3%/Lv) -&gt; +30% (L10)
+          <t>Accuracy: +15% (+1-2%/Lv) -&gt; +30%   |   Damage: +10% (+2-3%/Lv) -&gt; +30%
 Turns: 5 -&gt; 9   |   TP Cost: 5 (+2-3/Lv) -&gt; 28</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Row Y022: effect 31 added, 3 points of critical rate a level</t>
+          <t>Row Y022: effect 191 added, damage +10% to +30%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
balance: Mace Mastery x1.875 of vanilla, ATK and RES of the mace
The bonus multiplies the RES of the mace as well, and a healer heals by
her RES. Priest's Mace at C31, 400 battles: RES 107 to 117, heal per cast
178 to 190, won fights 16.7 to 16.4. A mace with no RES gains ATK only.
</commit_message>
<xml_diff>
--- a/data_tables/balance_skill_text.xlsx
+++ b/data_tables/balance_skill_text.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1272,6 +1272,38 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>PassiveSkillData_0244.bin</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Mace Mastery</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>ATK and RES bonus with mace equipped.</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>ATK and RES bonus: 5.6% -&gt; 9.4 -&gt; 13.1 -&gt; 16.9 -&gt; 18.8 -&gt; 20.6 -&gt; 22.5 -&gt; 24.4 -&gt; 26.3 -&gt; 28.1%</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Rows K114 - K123: the bonus reaches the RES of the mace as well (docs/FORMULAS.md 12.17)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
balance: Knock Down parries at any range, rates x1.875 of vanilla
The passive gains effect 250 (Counter, short and mid range) beside effect 305 (long range), with the same rates, 18.8% to 56.2% by level. Over the 40 bosses of the story the Mistress takes 15% less damage (1085 to 925 per battle); in the skill battery the skill moves from dead to niche. The reader of the variant keeps only the levels of the skill for an added effect. The level line of Mace Mastery is shortened to the 85 characters of a box line.
</commit_message>
<xml_diff>
--- a/data_tables/balance_skill_text.xlsx
+++ b/data_tables/balance_skill_text.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1295,12 +1295,44 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>ATK and RES bonus: 5.6% -&gt; 9.4 -&gt; 13.1 -&gt; 16.9 -&gt; 18.8 -&gt; 20.6 -&gt; 22.5 -&gt; 24.4 -&gt; 26.3 -&gt; 28.1%</t>
+          <t>ATK/RES: 5.6% -&gt; 9.4 -&gt; 13.1 -&gt; 16.9 -&gt; 18.8 -&gt; 20.6 -&gt; 22.5 -&gt; 24.4 -&gt; 26.3 -&gt; 28.1%</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
           <t>Rows K114 - K123: the bonus reaches the RES of the mace as well (docs/FORMULAS.md 12.17)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>PassiveSkillData_0264.bin</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Knock Down</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Occasionally parry and counterattack hits of any range.</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Activation rate: 18.8% -&gt; 28.1 -&gt; 37.5 -&gt; 46.9 -&gt; 56.2%</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Rows K056 - K060, Y023: rates x1.875 of vanilla, effect 250 added</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
balance: Life Bringer deals 8% to 16% of the max HP of the target
Effect 138 added beside the cut of max HP. The cut alone never removed current HP, since the blow had already taken more than the cut, so the skill did not shorten a fight. Used on the first turn only, over 16 bosses: won fights 6.8% shorter, no boss hurt; used on every turn it is 2.2% shorter and hurts 6 bosses.
</commit_message>
<xml_diff>
--- a/data_tables/balance_skill_text.xlsx
+++ b/data_tables/balance_skill_text.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1336,6 +1336,39 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Technique</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>TechniqueSkillData_0091.bin</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Life Bringer</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Short-range. Damage by enemy max HP and reduce its max HP.</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Max HP damage: 8% -&gt; 10% -&gt; 12% -&gt; 14% -&gt; 16% (L1-5 Max)   |   ATK: 110% -&gt; 150%
+Max HP reduction: 50% -&gt; 100%   |   TP Cost: 15 -&gt; 25   |   Speed: 0.85x</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Row Y024: effect 138 added; rows X056 - X060: ATK 110% to 150%</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
balance: Protect casts fast and cuts physical damage 15% to 30%
Chant factor 1.25 to 3.0 and speed factor x1.6 (2.0 to 2.25), and effect 179 (the cut of Material Guard, while the caster wears a shield) added beside the DEF. The TP cost is kept. With the tank buffing herself under Provoke: fights 7.6% longer instead of 16.2%, HP left of the party +1.0, 9 of 16 bosses hurt instead of 14, 3 served instead of 0.
</commit_message>
<xml_diff>
--- a/data_tables/balance_skill_text.xlsx
+++ b/data_tables/balance_skill_text.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1369,6 +1369,39 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Magic</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>MagicSkillData_0194.bin</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Protect</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Shield skill. Raise an ally's DEF and cut physical damage.</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>DEF: +20% -&gt; +28 -&gt; +36 -&gt; +44 -&gt; +50%   |   Damage reduction: 15% -&gt; 19 -&gt; 23 -&gt; 27 -&gt; 30%
+Turns: 5 -&gt; 9   |   TP Cost: 9 -&gt; 17   |   Speed: 2x -&gt; 2.25x   |   Chant: 3x</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Rows X066 - X070, Y025 - Y035: effect 179 added, quick cast</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>